<commit_message>
feat(train+data): add BTRXD pipeline updates, HF text embedding
</commit_message>
<xml_diff>
--- a/datasets/BTRXD_tumor_l100/Test_Folder/Test_text.xlsx
+++ b/datasets/BTRXD_tumor_l100/Test_Folder/Test_text.xlsx
@@ -443,3360 +443,3360 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IMG000736.png</t>
+          <t>IMG000024.png</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IMG001140.png</t>
+          <t>IMG000027.png</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; pelvis; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IMG001311.png</t>
+          <t>IMG000034.png</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; upper limb; humerus; oblique</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IMG001770.png</t>
+          <t>IMG000042.png</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IMG001289.png</t>
+          <t>IMG000046.png</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; fibula; lateral</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IMG001008.png</t>
+          <t>IMG000047.png</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IMG001528.png</t>
+          <t>IMG000051.png</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>IMG001193.png</t>
+          <t>IMG000054.png</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IMG000400.png</t>
+          <t>IMG000068.png</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>IMG001252.png</t>
+          <t>IMG000077.png</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>IMG001593.png</t>
+          <t>IMG000078.png</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>IMG000253.png</t>
+          <t>IMG000090.png</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IMG001604.png</t>
+          <t>IMG000093.png</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IMG001031.png</t>
+          <t>IMG000113.png</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IMG000619.png</t>
+          <t>IMG000118.png</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IMG001803.png</t>
+          <t>IMG000121.png</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; upper limb; humerus; oblique</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IMG000913.png</t>
+          <t>IMG000126.png</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IMG001799.png</t>
+          <t>IMG000138.png</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IMG000788.png</t>
+          <t>IMG000139.png</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; upper limb; radius; frontal</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>IMG000799.png</t>
+          <t>IMG000141.png</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>IMG001844.png</t>
+          <t>IMG000147.png</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>IMG001079.png</t>
+          <t>IMG000152.png</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; pelvis; hip bone; frontal</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>IMG000857.png</t>
+          <t>IMG000154.png</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>IMG001820.png</t>
+          <t>IMG000155.png</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; pelvis; hip bone; frontal</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IMG001339.png</t>
+          <t>IMG000160.png</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; pelvis; femur; oblique</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IMG001787.png</t>
+          <t>IMG000161.png</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; pelvis; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IMG001117.png</t>
+          <t>IMG000170.png</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IMG000448.png</t>
+          <t>IMG000173.png</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; upper limb; radius; frontal</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IMG000395.png</t>
+          <t>IMG000178.png</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IMG001497.png</t>
+          <t>IMG000180.png</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; oblique</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>IMG000304.png</t>
+          <t>IMG000195.png</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IMG001297.png</t>
+          <t>IMG000204.png</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IMG001790.png</t>
+          <t>IMG000205.png</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>IMG000944.png</t>
+          <t>IMG000224.png</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>IMG000967.png</t>
+          <t>IMG000225.png</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>IMG000430.png</t>
+          <t>IMG000228.png</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IMG001728.png</t>
+          <t>IMG000229.png</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IMG000764.png</t>
+          <t>IMG000247.png</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; pelvis; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IMG000815.png</t>
+          <t>IMG000253.png</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>IMG001065.png</t>
+          <t>IMG000255.png</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>IMG001825.png</t>
+          <t>IMG000258.png</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IMG000864.png</t>
+          <t>IMG000283.png</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IMG001066.png</t>
+          <t>IMG000287.png</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; frontal</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IMG001285.png</t>
+          <t>IMG000292.png</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IMG000643.png</t>
+          <t>IMG000304.png</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; oblique</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IMG001010.png</t>
+          <t>IMG000308.png</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>IMG001039.png</t>
+          <t>IMG000311.png</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IMG001283.png</t>
+          <t>IMG000316.png</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; oblique</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IMG000614.png</t>
+          <t>IMG000317.png</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; lateral</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>IMG001791.png</t>
+          <t>IMG000319.png</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IMG000645.png</t>
+          <t>IMG000328.png</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>IMG000435.png</t>
+          <t>IMG000334.png</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>IMG000903.png</t>
+          <t>IMG000336.png</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>IMG001142.png</t>
+          <t>IMG000344.png</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>IMG001585.png</t>
+          <t>IMG000361.png</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>IMG001527.png</t>
+          <t>IMG000366.png</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; oblique</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>IMG000812.png</t>
+          <t>IMG000369.png</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>IMG000951.png</t>
+          <t>IMG000383.png</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; frontal</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>IMG001158.png</t>
+          <t>IMG000387.png</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; lateral</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>IMG000544.png</t>
+          <t>IMG000395.png</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur, hip bone; frontal</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>IMG000705.png</t>
+          <t>IMG000400.png</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>IMG001806.png</t>
+          <t>IMG000415.png</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>IMG001516.png</t>
+          <t>IMG000430.png</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>IMG001045.png</t>
+          <t>IMG000431.png</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>IMG001656.png</t>
+          <t>IMG000435.png</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>IMG001584.png</t>
+          <t>IMG000437.png</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; radius; frontal</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>IMG000543.png</t>
+          <t>IMG000438.png</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; radius; lateral</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>IMG000336.png</t>
+          <t>IMG000446.png</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; pelvis; hip bone; frontal</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>IMG000648.png</t>
+          <t>IMG000448.png</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>IMG000817.png</t>
+          <t>IMG000455.png</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>IMG000706.png</t>
+          <t>IMG000457.png</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>IMG001358.png</t>
+          <t>IMG000465.png</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>IMG000283.png</t>
+          <t>IMG000477.png</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>IMG001411.png</t>
+          <t>IMG000482.png</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>IMG000582.png</t>
+          <t>IMG000489.png</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; oblique</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>IMG000319.png</t>
+          <t>IMG000499.png</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; lateral</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>IMG001320.png</t>
+          <t>IMG000501.png</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>IMG001310.png</t>
+          <t>IMG000509.png</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>IMG001457.png</t>
+          <t>IMG000522.png</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; lateral</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>IMG000716.png</t>
+          <t>IMG000523.png</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; frontal</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>IMG001198.png</t>
+          <t>IMG000529.png</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; oblique</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>IMG000567.png</t>
+          <t>IMG000530.png</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>IMG001035.png</t>
+          <t>IMG000533.png</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; oblique</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>IMG001804.png</t>
+          <t>IMG000539.png</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>IMG001139.png</t>
+          <t>IMG000543.png</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>IMG001603.png</t>
+          <t>IMG000544.png</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>IMG000650.png</t>
+          <t>IMG000549.png</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; lateral</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>IMG000785.png</t>
+          <t>IMG000567.png</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>IMG000907.png</t>
+          <t>IMG000576.png</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>IMG000465.png</t>
+          <t>IMG000582.png</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; oblique</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>IMG000612.png</t>
+          <t>IMG000608.png</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>malignant; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>IMG001260.png</t>
+          <t>IMG000612.png</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>IMG000998.png</t>
+          <t>IMG000614.png</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>IMG000477.png</t>
+          <t>IMG000617.png</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>IMG001131.png</t>
+          <t>IMG000619.png</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>IMG001094.png</t>
+          <t>IMG000622.png</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; pelvis; hip bone; frontal</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>IMG000344.png</t>
+          <t>IMG000623.png</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; pelvis; hip bone; oblique</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>IMG001147.png</t>
+          <t>IMG000634.png</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; oblique</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>IMG001196.png</t>
+          <t>IMG000643.png</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; lateral</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>IMG001645.png</t>
+          <t>IMG000645.png</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>IMG001227.png</t>
+          <t>IMG000647.png</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>IMG000647.png</t>
+          <t>IMG000648.png</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>IMG001177.png</t>
+          <t>IMG000650.png</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; knee-joint; frontal</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>IMG000539.png</t>
+          <t>IMG000660.png</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>IMG001236.png</t>
+          <t>IMG000678.png</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; lateral</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>IMG001277.png</t>
+          <t>IMG000701.png</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>IMG000717.png</t>
+          <t>IMG000705.png</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; lateral</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>IMG001261.png</t>
+          <t>IMG000706.png</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>IMG001563.png</t>
+          <t>IMG000710.png</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; oblique</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>IMG001819.png</t>
+          <t>IMG000716.png</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>IMG001813.png</t>
+          <t>IMG000717.png</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>IMG000522.png</t>
+          <t>IMG000736.png</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>IMG001832.png</t>
+          <t>IMG000764.png</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>IMG000457.png</t>
+          <t>IMG000773.png</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; lateral</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>IMG001060.png</t>
+          <t>IMG000785.png</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>IMG000897.png</t>
+          <t>IMG000788.png</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>IMG000369.png</t>
+          <t>IMG000791.png</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; pelvis; femur; oblique</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>IMG000431.png</t>
+          <t>IMG000798.png</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>IMG000798.png</t>
+          <t>IMG000799.png</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>IMG001254.png</t>
+          <t>IMG000812.png</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>IMG001068.png</t>
+          <t>IMG000814.png</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IMG000455.png</t>
+          <t>IMG000815.png</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>IMG001299.png</t>
+          <t>IMG000817.png</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>IMG000617.png</t>
+          <t>IMG000834.png</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; pelvis; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>IMG001591.png</t>
+          <t>IMG000838.png</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; pelvis; hip bone; frontal</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>IMG000361.png</t>
+          <t>IMG000839.png</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; radius; frontal</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>IMG000993.png</t>
+          <t>IMG000857.png</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; lateral</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>IMG001205.png</t>
+          <t>IMG000864.png</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>IMG001246.png</t>
+          <t>IMG000866.png</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>IMG000509.png</t>
+          <t>IMG000868.png</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>IMG001302.png</t>
+          <t>IMG000876.png</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>IMG000499.png</t>
+          <t>IMG000882.png</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>IMG001847.png</t>
+          <t>IMG000888.png</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>IMG001182.png</t>
+          <t>IMG000897.png</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>IMG000866.png</t>
+          <t>IMG000903.png</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>IMG000701.png</t>
+          <t>IMG000907.png</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>IMG001824.png</t>
+          <t>IMG000910.png</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>IMG001191.png</t>
+          <t>IMG000913.png</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>IMG001465.png</t>
+          <t>IMG000936.png</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>IMG000710.png</t>
+          <t>IMG000941.png</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; ulna, radius; frontal</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>IMG000255.png</t>
+          <t>IMG000944.png</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>IMG001034.png</t>
+          <t>IMG000951.png</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; lateral</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>IMG001550.png</t>
+          <t>IMG000965.png</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; ulna; frontal</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>IMG000882.png</t>
+          <t>IMG000966.png</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>IMG001451.png</t>
+          <t>IMG000967.png</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>IMG000814.png</t>
+          <t>IMG000975.png</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; frontal</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>IMG000311.png</t>
+          <t>IMG000993.png</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>IMG001789.png</t>
+          <t>IMG000998.png</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>IMG000910.png</t>
+          <t>IMG001008.png</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>IMG000876.png</t>
+          <t>IMG001010.png</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>IMG000501.png</t>
+          <t>IMG001028.png</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>IMG000328.png</t>
+          <t>IMG001031.png</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>IMG000334.png</t>
+          <t>IMG001034.png</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>IMG001464.png</t>
+          <t>IMG001035.png</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>IMG000482.png</t>
+          <t>IMG001039.png</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>IMG000530.png</t>
+          <t>IMG001045.png</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>IMG000660.png</t>
+          <t>IMG001056.png</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; pelvis; hip bone; frontal</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>IMG000888.png</t>
+          <t>IMG001060.png</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>IMG000936.png</t>
+          <t>IMG001065.png</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>IMG001028.png</t>
+          <t>IMG001066.png</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>IMG000308.png</t>
+          <t>IMG001068.png</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>IMG000576.png</t>
+          <t>IMG001079.png</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>benign bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>IMG001056.png</t>
+          <t>IMG001094.png</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>IMG000247.png</t>
+          <t>IMG001114.png</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; upper limb; radius; frontal</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>IMG000622.png</t>
+          <t>IMG001115.png</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; upper limb; radius; lateral</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>IMG001596.png</t>
+          <t>IMG001117.png</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>IMG001805.png</t>
+          <t>IMG001127.png</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; upper limb; shoulder-joint; oblique</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>IMG000838.png</t>
+          <t>IMG001131.png</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; lower limb; knee-joint; frontal</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>IMG000623.png</t>
+          <t>IMG001139.png</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>IMG000834.png</t>
+          <t>IMG001140.png</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>IMG000791.png</t>
+          <t>IMG001142.png</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>IMG000446.png</t>
+          <t>IMG001147.png</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>IMG001473.png</t>
+          <t>IMG001158.png</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>benign bone tumor, pelvis.</t>
+          <t>benign; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>IMG000317.png</t>
+          <t>IMG001170.png</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; hand; frontal</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>IMG000287.png</t>
+          <t>IMG001177.png</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>IMG000868.png</t>
+          <t>IMG001182.png</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; knee-joint; frontal</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>IMG000549.png</t>
+          <t>IMG001188.png</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; radius; frontal</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>IMG001267.png</t>
+          <t>IMG001191.png</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; knee-joint; lateral</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>IMG001811.png</t>
+          <t>IMG001193.png</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>IMG000437.png</t>
+          <t>IMG001196.png</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; knee-joint; frontal</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>IMG001243.png</t>
+          <t>IMG001198.png</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; knee-joint; lateral</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>IMG000415.png</t>
+          <t>IMG001205.png</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; knee-joint; lateral</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>IMG000634.png</t>
+          <t>IMG001227.png</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>IMG000839.png</t>
+          <t>IMG001236.png</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; knee-joint; frontal</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>IMG001680.png</t>
+          <t>IMG001243.png</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; ulna, radius; frontal</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>IMG000678.png</t>
+          <t>IMG001246.png</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>IMG000366.png</t>
+          <t>IMG001249.png</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; radius; lateral</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>IMG001668.png</t>
+          <t>IMG001252.png</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>IMG001855.png</t>
+          <t>IMG001254.png</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; fibula; lateral</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>IMG001494.png</t>
+          <t>IMG001260.png</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>IMG001381.png</t>
+          <t>IMG001261.png</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>IMG001677.png</t>
+          <t>IMG001267.png</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>IMG001857.png</t>
+          <t>IMG001277.png</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>IMG001114.png</t>
+          <t>IMG001283.png</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia, fibula; lateral</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>IMG001485.png</t>
+          <t>IMG001285.png</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>IMG000965.png</t>
+          <t>IMG001289.png</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; femur, hip bone; oblique</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>IMG000387.png</t>
+          <t>IMG001292.png</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; hand; oblique</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>IMG001723.png</t>
+          <t>IMG001297.png</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>IMG001170.png</t>
+          <t>IMG001299.png</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>IMG001676.png</t>
+          <t>IMG001302.png</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>IMG000975.png</t>
+          <t>IMG001310.png</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>IMG000773.png</t>
+          <t>IMG001311.png</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>IMG001357.png</t>
+          <t>IMG001320.png</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>IMG000383.png</t>
+          <t>IMG001339.png</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>IMG000533.png</t>
+          <t>IMG001357.png</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>IMG001743.png</t>
+          <t>IMG001358.png</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>IMG001188.png</t>
+          <t>IMG001361.png</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>IMG000523.png</t>
+          <t>IMG001373.png</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>malignant; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>IMG000258.png</t>
+          <t>IMG001381.png</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>IMG001292.png</t>
+          <t>IMG001400.png</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; ulna; lateral</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>IMG001461.png</t>
+          <t>IMG001405.png</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>IMG001839.png</t>
+          <t>IMG001409.png</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>IMG001249.png</t>
+          <t>IMG001411.png</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; femur; oblique</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>IMG000438.png</t>
+          <t>IMG001413.png</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>malignant; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>IMG000966.png</t>
+          <t>IMG001451.png</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>IMG001636.png</t>
+          <t>IMG001457.png</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>IMG001405.png</t>
+          <t>IMG001461.png</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; ulna; lateral</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>IMG000489.png</t>
+          <t>IMG001464.png</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia, fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>IMG000292.png</t>
+          <t>IMG001465.png</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia, fibula; lateral</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>IMG001400.png</t>
+          <t>IMG001473.png</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; pelvis; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>IMG000529.png</t>
+          <t>IMG001475.png</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>malignant; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>IMG001739.png</t>
+          <t>IMG001485.png</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>IMG001751.png</t>
+          <t>IMG001494.png</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; upper limb; radius; frontal</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>IMG001127.png</t>
+          <t>IMG001497.png</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>IMG001115.png</t>
+          <t>IMG001516.png</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>IMG001848.png</t>
+          <t>IMG001521.png</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>malignant; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>IMG001361.png</t>
+          <t>IMG001527.png</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>IMG000941.png</t>
+          <t>IMG001528.png</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>IMG000316.png</t>
+          <t>IMG001534.png</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>benign bone tumor, upper limb.</t>
+          <t>malignant; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>IMG001373.png</t>
+          <t>IMG001535.png</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>IMG001535.png</t>
+          <t>IMG001550.png</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>IMG000225.png</t>
+          <t>IMG001563.png</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>IMG000180.png</t>
+          <t>IMG001584.png</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; ankle-joint; lateral</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>IMG001626.png</t>
+          <t>IMG001585.png</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; ankle-joint; frontal</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>IMG000228.png</t>
+          <t>IMG001591.png</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia, fibula, femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>IMG000113.png</t>
+          <t>IMG001593.png</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>IMG001534.png</t>
+          <t>IMG001596.png</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; pelvis; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>IMG000054.png</t>
+          <t>IMG001603.png</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>IMG000147.png</t>
+          <t>IMG001604.png</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>IMG000224.png</t>
+          <t>IMG001626.png</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>malignant; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>IMG000138.png</t>
+          <t>IMG001636.png</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; upper limb; ulna, radius, humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>IMG000047.png</t>
+          <t>IMG001645.png</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>IMG000093.png</t>
+          <t>IMG001656.png</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; lateral</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>IMG000195.png</t>
+          <t>IMG001668.png</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; oblique</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>IMG001409.png</t>
+          <t>IMG001674.png</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>malignant; upper limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>IMG000068.png</t>
+          <t>IMG001676.png</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; frontal</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>IMG000090.png</t>
+          <t>IMG001677.png</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; oblique</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>IMG000205.png</t>
+          <t>IMG001680.png</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>IMG000229.png</t>
+          <t>IMG001723.png</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; oblique</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>IMG000046.png</t>
+          <t>IMG001728.png</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>IMG001866.png</t>
+          <t>IMG001739.png</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>IMG000126.png</t>
+          <t>IMG001740.png</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>malignant; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>IMG000608.png</t>
+          <t>IMG001741.png</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>malignant; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>IMG000118.png</t>
+          <t>IMG001743.png</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; frontal</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>IMG000024.png</t>
+          <t>IMG001751.png</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; upper limb; hand; frontal</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>IMG001475.png</t>
+          <t>IMG001764.png</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>malignant; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>IMG001740.png</t>
+          <t>IMG001770.png</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>IMG000178.png</t>
+          <t>IMG001787.png</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>IMG001521.png</t>
+          <t>IMG001789.png</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; lateral</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>IMG001413.png</t>
+          <t>IMG001790.png</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; fibula; frontal</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>IMG001741.png</t>
+          <t>IMG001791.png</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>IMG000141.png</t>
+          <t>IMG001799.png</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; tibia; lateral</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>IMG000170.png</t>
+          <t>IMG001803.png</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>malignant bone tumor, lower limb.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>IMG000027.png</t>
+          <t>IMG001804.png</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>malignant bone tumor, pelvis.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>IMG000155.png</t>
+          <t>IMG001805.png</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>malignant bone tumor, pelvis.</t>
+          <t>benign; pelvis; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>IMG000152.png</t>
+          <t>IMG001806.png</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>malignant bone tumor, pelvis.</t>
+          <t>benign; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>IMG000160.png</t>
+          <t>IMG001811.png</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>malignant bone tumor, pelvis.</t>
+          <t>benign; upper limb; humerus; oblique</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>IMG000161.png</t>
+          <t>IMG001813.png</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>malignant bone tumor, pelvis.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>IMG000173.png</t>
+          <t>IMG001819.png</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>IMG000077.png</t>
+          <t>IMG001820.png</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; lower limb; fibula, femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>IMG000042.png</t>
+          <t>IMG001824.png</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>IMG001764.png</t>
+          <t>IMG001825.png</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>IMG000078.png</t>
+          <t>IMG001832.png</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; lower limb; tibia; frontal</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>IMG000121.png</t>
+          <t>IMG001839.png</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>IMG000139.png</t>
+          <t>IMG001844.png</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; lower limb; foot; frontal</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>IMG000204.png</t>
+          <t>IMG001847.png</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; lower limb; femur; frontal</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>IMG001674.png</t>
+          <t>IMG001848.png</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>IMG000051.png</t>
+          <t>IMG001855.png</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; upper limb; humerus; frontal</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>IMG000154.png</t>
+          <t>IMG001857.png</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>benign; upper limb; ulna; frontal</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>IMG000034.png</t>
+          <t>IMG001866.png</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>malignant bone tumor, upper limb.</t>
+          <t>malignant; lower limb; femur; lateral</t>
         </is>
       </c>
     </row>

</xml_diff>